<commit_message>
fix: refine Ziraat building document export
</commit_message>
<xml_diff>
--- a/templates/ziraat-ek-tablo.xlsx
+++ b/templates/ziraat-ek-tablo.xlsx
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B3" s="113" t="inlineStr">
         <is>
-          <t>{{TASINMAZ_ID}}</t>
+          <t>Sistemden BKNZ</t>
         </is>
       </c>
       <c r="C3" s="113" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="D3" s="113" t="inlineStr">
         <is>
-          <t>{{YAPI_RUHSATI}}</t>
+          <t>{{YAPI_BELGESI}}</t>
         </is>
       </c>
       <c r="E3" s="113" t="n">
@@ -2655,11 +2655,7 @@
       <c r="A4" s="121" t="n"/>
       <c r="B4" s="122" t="n"/>
       <c r="C4" s="122" t="n"/>
-      <c r="D4" s="122" t="inlineStr">
-        <is>
-          <t>{{ISKAN_BELGESI}}</t>
-        </is>
-      </c>
+      <c r="D4" s="122" t="n"/>
       <c r="E4" s="122" t="n"/>
       <c r="F4" s="123" t="n"/>
       <c r="G4" s="124" t="n"/>
@@ -2763,10 +2759,9 @@
         <f>C3</f>
         <v/>
       </c>
-      <c r="D10" s="118" t="inlineStr">
-        <is>
-          <t>{{YAPI_RUHSATI}}</t>
-        </is>
+      <c r="D10" s="118">
+        <f>D3</f>
+        <v/>
       </c>
       <c r="E10" s="116" t="n">
         <v>0</v>
@@ -2792,11 +2787,7 @@
         <f>C4</f>
         <v/>
       </c>
-      <c r="D11" s="122" t="inlineStr">
-        <is>
-          <t>{{ISKAN_BELGESI}}</t>
-        </is>
-      </c>
+      <c r="D11" s="122" t="n"/>
       <c r="E11" s="122">
         <f>E4</f>
         <v/>
@@ -2973,7 +2964,7 @@
       </c>
       <c r="B3" s="66" t="inlineStr">
         <is>
-          <t>{{TASINMAZ_ID}}</t>
+          <t>Sistemden BKNZ</t>
         </is>
       </c>
       <c r="C3" s="67" t="inlineStr">
@@ -3032,7 +3023,7 @@
       </c>
       <c r="F4" s="60" t="inlineStr">
         <is>
-          <t>{{YAPI_RUHSATI}}</t>
+          <t>{{YAPI_BELGESI}}</t>
         </is>
       </c>
       <c r="G4" s="60" t="n">

</xml_diff>

<commit_message>
feat: Ziraat ek tablo two-decimal display, adjacent-order KAKS, NİTELİKLİ totals
Per the user's five corrections:

- Area, per-m² unit value, Hmax and post-setback parcel size cells now use
  the #,##0.00 number format (was #,##0), including the total rows, so 192.74
  no longer rounds to 193. The stored value stays raw; two decimals are only
  the cell format.
- ARSA F3 (KAKS/Emsal) is filled via a ZRT_KAKS_OR_FLOOR resolver: when the
  building order is bitişik it writes the floor count, otherwise KAKS —
  matching composeImarCalculatedEmsal's precedence.
- NİTELİKLİ GAYRİMENKUL totals fixed to G9 =SUM(G4:G8) and G18 =SUM(G14:G17)
  so the arsa row is excluded from the sum.

Verified via npm run verify and end-to-end in a live browser (192.74 kept,
adjacent order yields the floor count, other orders yield KAKS).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/ziraat-ek-tablo.xlsx
+++ b/templates/ziraat-ek-tablo.xlsx
@@ -689,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1050,6 +1050,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1057,11 +1060,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1635,12 +1653,12 @@
           <t>{{PARSEL}}</t>
         </is>
       </c>
-      <c r="D3" s="116" t="inlineStr">
+      <c r="D3" s="122" t="inlineStr">
         <is>
           <t>{{LAND_AREA}}</t>
         </is>
       </c>
-      <c r="E3" s="97">
+      <c r="E3" s="98">
         <f>F3/D3</f>
         <v/>
       </c>
@@ -1661,7 +1679,7 @@
           <t>SARI İLE BOYALI ALANLARA GİRİŞ YAPILMALIDIR</t>
         </is>
       </c>
-      <c r="K3" s="122" t="n"/>
+      <c r="K3" s="123" t="n"/>
     </row>
     <row r="4" ht="34.5" customHeight="1">
       <c r="A4" s="100" t="n"/>
@@ -1673,8 +1691,8 @@
       <c r="G4" s="104" t="n"/>
       <c r="H4" s="85" t="n"/>
       <c r="I4" s="85" t="n"/>
-      <c r="J4" s="123" t="n"/>
-      <c r="K4" s="124" t="n"/>
+      <c r="J4" s="124" t="n"/>
+      <c r="K4" s="125" t="n"/>
     </row>
     <row r="5" ht="34.5" customHeight="1" thickBot="1">
       <c r="A5" s="32" t="n"/>
@@ -1686,8 +1704,8 @@
       <c r="G5" s="35" t="n"/>
       <c r="H5" s="85" t="n"/>
       <c r="I5" s="85" t="n"/>
-      <c r="J5" s="125" t="n"/>
-      <c r="K5" s="126" t="n"/>
+      <c r="J5" s="126" t="n"/>
+      <c r="K5" s="127" t="n"/>
     </row>
     <row r="6" ht="34.5" customHeight="1">
       <c r="A6" s="32" t="n"/>
@@ -1723,7 +1741,7 @@
       </c>
       <c r="B8" s="120" t="n"/>
       <c r="C8" s="120" t="n"/>
-      <c r="D8" s="36">
+      <c r="D8" s="45">
         <f>SUM(D3:D7)</f>
         <v/>
       </c>
@@ -1826,11 +1844,11 @@
         <f>C3</f>
         <v/>
       </c>
-      <c r="D12" s="97">
+      <c r="D12" s="98">
         <f>D3</f>
         <v/>
       </c>
-      <c r="E12" s="97">
+      <c r="E12" s="98">
         <f>F12/D12</f>
         <v/>
       </c>
@@ -1909,7 +1927,7 @@
       </c>
       <c r="B17" s="120" t="n"/>
       <c r="C17" s="120" t="n"/>
-      <c r="D17" s="36">
+      <c r="D17" s="45">
         <f>SUM(D12:D16)</f>
         <v/>
       </c>
@@ -1974,16 +1992,16 @@
           <t>ARSA İMAR VE YAPILAŞMA KOŞULLARI</t>
         </is>
       </c>
-      <c r="B1" s="127" t="n"/>
-      <c r="C1" s="127" t="n"/>
-      <c r="D1" s="127" t="n"/>
-      <c r="E1" s="127" t="n"/>
-      <c r="F1" s="127" t="n"/>
-      <c r="G1" s="127" t="n"/>
-      <c r="H1" s="127" t="n"/>
-      <c r="I1" s="127" t="n"/>
-      <c r="J1" s="127" t="n"/>
-      <c r="K1" s="128" t="n"/>
+      <c r="B1" s="128" t="n"/>
+      <c r="C1" s="128" t="n"/>
+      <c r="D1" s="128" t="n"/>
+      <c r="E1" s="128" t="n"/>
+      <c r="F1" s="128" t="n"/>
+      <c r="G1" s="128" t="n"/>
+      <c r="H1" s="128" t="n"/>
+      <c r="I1" s="128" t="n"/>
+      <c r="J1" s="128" t="n"/>
+      <c r="K1" s="129" t="n"/>
       <c r="L1" s="85" t="n"/>
       <c r="M1" s="85" t="n"/>
       <c r="N1" s="85" t="n"/>
@@ -2066,7 +2084,7 @@
           <t>{{PARSEL}}</t>
         </is>
       </c>
-      <c r="D3" s="116" t="inlineStr">
+      <c r="D3" s="122" t="inlineStr">
         <is>
           <t>{{LAND_AREA}}</t>
         </is>
@@ -2082,7 +2100,7 @@
       <c r="G3" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="96" t="n">
+      <c r="H3" s="98" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="119" t="inlineStr">
@@ -2090,7 +2108,7 @@
           <t>{{CALCULATED_EMSAL}}</t>
         </is>
       </c>
-      <c r="J3" s="119" t="inlineStr">
+      <c r="J3" s="130" t="inlineStr">
         <is>
           <t>{{POST_ROAD_SETBACK_PARCEL_AREA}}</t>
         </is>
@@ -2173,7 +2191,7 @@
       </c>
       <c r="B8" s="120" t="n"/>
       <c r="C8" s="121" t="n"/>
-      <c r="D8" s="36">
+      <c r="D8" s="45">
         <f>SUM(D3:D7)</f>
         <v/>
       </c>
@@ -2212,12 +2230,12 @@
           <t>ARSA YASAL DURUM DEĞERİ/KANAAT TABLOSU</t>
         </is>
       </c>
-      <c r="B10" s="129" t="n"/>
-      <c r="C10" s="129" t="n"/>
-      <c r="D10" s="129" t="n"/>
-      <c r="E10" s="129" t="n"/>
-      <c r="F10" s="129" t="n"/>
-      <c r="G10" s="130" t="n"/>
+      <c r="B10" s="131" t="n"/>
+      <c r="C10" s="131" t="n"/>
+      <c r="D10" s="131" t="n"/>
+      <c r="E10" s="131" t="n"/>
+      <c r="F10" s="131" t="n"/>
+      <c r="G10" s="132" t="n"/>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
@@ -2285,12 +2303,12 @@
         <f>C3</f>
         <v/>
       </c>
-      <c r="D12" s="116" t="inlineStr">
+      <c r="D12" s="122" t="inlineStr">
         <is>
           <t>{{LAND_AREA}}</t>
         </is>
       </c>
-      <c r="E12" s="102">
+      <c r="E12" s="103">
         <f>F12/D12</f>
         <v/>
       </c>
@@ -2387,9 +2405,9 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B17" s="131" t="n"/>
-      <c r="C17" s="132" t="n"/>
-      <c r="D17" s="50">
+      <c r="B17" s="133" t="n"/>
+      <c r="C17" s="134" t="n"/>
+      <c r="D17" s="51">
         <f>SUM(D12:D16)</f>
         <v/>
       </c>
@@ -2428,12 +2446,12 @@
           <t>ARSA MEVCUT DURUM DEĞERİ/KANAAT TABLOSU</t>
         </is>
       </c>
-      <c r="B19" s="129" t="n"/>
-      <c r="C19" s="129" t="n"/>
-      <c r="D19" s="129" t="n"/>
-      <c r="E19" s="129" t="n"/>
-      <c r="F19" s="129" t="n"/>
-      <c r="G19" s="130" t="n"/>
+      <c r="B19" s="131" t="n"/>
+      <c r="C19" s="131" t="n"/>
+      <c r="D19" s="131" t="n"/>
+      <c r="E19" s="131" t="n"/>
+      <c r="F19" s="131" t="n"/>
+      <c r="G19" s="132" t="n"/>
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
@@ -2504,11 +2522,11 @@
         <f>C3</f>
         <v/>
       </c>
-      <c r="D21" s="33">
+      <c r="D21" s="39">
         <f>D3</f>
         <v/>
       </c>
-      <c r="E21" s="34">
+      <c r="E21" s="39">
         <f>F21/D21</f>
         <v/>
       </c>
@@ -2604,9 +2622,9 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B26" s="131" t="n"/>
-      <c r="C26" s="132" t="n"/>
-      <c r="D26" s="50">
+      <c r="B26" s="133" t="n"/>
+      <c r="C26" s="134" t="n"/>
+      <c r="D26" s="51">
         <f>SUM(D21:D25)</f>
         <v/>
       </c>
@@ -2669,12 +2687,12 @@
           <t>KONUT - İŞYERLERİ YASAL DURUM DEĞERİ</t>
         </is>
       </c>
-      <c r="B1" s="127" t="n"/>
-      <c r="C1" s="127" t="n"/>
-      <c r="D1" s="127" t="n"/>
-      <c r="E1" s="127" t="n"/>
-      <c r="F1" s="127" t="n"/>
-      <c r="G1" s="128" t="n"/>
+      <c r="B1" s="128" t="n"/>
+      <c r="C1" s="128" t="n"/>
+      <c r="D1" s="128" t="n"/>
+      <c r="E1" s="128" t="n"/>
+      <c r="F1" s="128" t="n"/>
+      <c r="G1" s="129" t="n"/>
       <c r="H1" s="85" t="n"/>
       <c r="I1" s="85" t="n"/>
       <c r="J1" s="85" t="n"/>
@@ -2739,12 +2757,12 @@
           <t>{{YAPI_BELGESI}}</t>
         </is>
       </c>
-      <c r="E3" s="38" t="inlineStr">
+      <c r="E3" s="135" t="inlineStr">
         <is>
           <t>{{TOTAL_LEGAL_AREA}}</t>
         </is>
       </c>
-      <c r="F3" s="31">
+      <c r="F3" s="135">
         <f>IFERROR(G3/E3,0)</f>
         <v/>
       </c>
@@ -2757,7 +2775,7 @@
           <t>SARI İLE BOYALI ALANLARA GİRİŞ YAPILMALIDIR</t>
         </is>
       </c>
-      <c r="J3" s="122" t="n"/>
+      <c r="J3" s="123" t="n"/>
     </row>
     <row r="4" ht="34.5" customHeight="1">
       <c r="A4" s="32" t="n"/>
@@ -2768,8 +2786,8 @@
       <c r="F4" s="34" t="n"/>
       <c r="G4" s="54" t="n"/>
       <c r="H4" s="85" t="n"/>
-      <c r="I4" s="123" t="n"/>
-      <c r="J4" s="124" t="n"/>
+      <c r="I4" s="124" t="n"/>
+      <c r="J4" s="125" t="n"/>
     </row>
     <row r="5" ht="34.5" customHeight="1" thickBot="1">
       <c r="A5" s="32" t="n"/>
@@ -2780,8 +2798,8 @@
       <c r="F5" s="34" t="n"/>
       <c r="G5" s="54" t="n"/>
       <c r="H5" s="85" t="n"/>
-      <c r="I5" s="125" t="n"/>
-      <c r="J5" s="126" t="n"/>
+      <c r="I5" s="126" t="n"/>
+      <c r="J5" s="127" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1" thickBot="1">
       <c r="A6" s="72" t="inlineStr">
@@ -2789,10 +2807,10 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B6" s="131" t="n"/>
-      <c r="C6" s="131" t="n"/>
-      <c r="D6" s="132" t="n"/>
-      <c r="E6" s="55">
+      <c r="B6" s="133" t="n"/>
+      <c r="C6" s="133" t="n"/>
+      <c r="D6" s="134" t="n"/>
+      <c r="E6" s="51">
         <f>SUM(E3:E5)</f>
         <v/>
       </c>
@@ -2893,12 +2911,12 @@
         <f>D3</f>
         <v/>
       </c>
-      <c r="E10" s="58" t="inlineStr">
+      <c r="E10" s="136" t="inlineStr">
         <is>
           <t>{{TOTAL_CURRENT_AREA}}</t>
         </is>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="135">
         <f>IFERROR(G10/E10,0)</f>
         <v/>
       </c>
@@ -2951,10 +2969,10 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B14" s="133" t="n"/>
-      <c r="C14" s="133" t="n"/>
-      <c r="D14" s="133" t="n"/>
-      <c r="E14" s="64">
+      <c r="B14" s="137" t="n"/>
+      <c r="C14" s="137" t="n"/>
+      <c r="D14" s="137" t="n"/>
+      <c r="E14" s="138">
         <f>SUM(E10:E13)</f>
         <v/>
       </c>
@@ -3109,12 +3127,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G3" s="116" t="inlineStr">
+      <c r="G3" s="122" t="inlineStr">
         <is>
           <t>{{LAND_AREA}}</t>
         </is>
       </c>
-      <c r="H3" s="109">
+      <c r="H3" s="139">
         <f>I3/G3</f>
         <v/>
       </c>
@@ -3157,12 +3175,12 @@
           <t>{{YAPI_BELGESI}}</t>
         </is>
       </c>
-      <c r="G4" s="114" t="inlineStr">
+      <c r="G4" s="122" t="inlineStr">
         <is>
           <t>{{TOTAL_LEGAL_AREA}}</t>
         </is>
       </c>
-      <c r="H4" s="109">
+      <c r="H4" s="139">
         <f>I4/G4</f>
         <v/>
       </c>
@@ -3257,13 +3275,13 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B9" s="133" t="n"/>
-      <c r="C9" s="133" t="n"/>
-      <c r="D9" s="133" t="n"/>
-      <c r="E9" s="133" t="n"/>
-      <c r="F9" s="134" t="n"/>
-      <c r="G9" s="65">
-        <f>SUM(G3:G8)</f>
+      <c r="B9" s="137" t="n"/>
+      <c r="C9" s="137" t="n"/>
+      <c r="D9" s="137" t="n"/>
+      <c r="E9" s="137" t="n"/>
+      <c r="F9" s="140" t="n"/>
+      <c r="G9" s="138">
+        <f>SUM(G4:G8)</f>
         <v/>
       </c>
       <c r="H9" s="65" t="n"/>
@@ -3394,12 +3412,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="116" t="inlineStr">
+      <c r="G13" s="122" t="inlineStr">
         <is>
           <t>{{LAND_AREA}}</t>
         </is>
       </c>
-      <c r="H13" s="109">
+      <c r="H13" s="139">
         <f>I13/G13</f>
         <v/>
       </c>
@@ -3445,7 +3463,7 @@
           <t>{{YAPI_BELGESI}}</t>
         </is>
       </c>
-      <c r="G14" s="114" t="inlineStr">
+      <c r="G14" s="122" t="inlineStr">
         <is>
           <t>{{TOTAL_CURRENT_AREA}}</t>
         </is>
@@ -3541,8 +3559,8 @@
       <c r="D18" s="120" t="n"/>
       <c r="E18" s="121" t="n"/>
       <c r="F18" s="46" t="n"/>
-      <c r="G18" s="46">
-        <f>SUM(G13:G17)</f>
+      <c r="G18" s="45">
+        <f>SUM(G14:G17)</f>
         <v/>
       </c>
       <c r="H18" s="36" t="n"/>

</xml_diff>